<commit_message>
Veepee : C0191-C0193 remplacés par V0891, V0732, V0913 (vrac 100 g, RRP 12 €), EAN et fiches complétés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/veepee/Veepee - stock disponible vente privee.xlsx
+++ b/veepee/Veepee - stock disponible vente privee.xlsx
@@ -5553,22 +5553,22 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>V0742</t>
+          <t>V0732</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>5413393800358</t>
+          <t>5413393800693</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Ange Gardien</t>
+          <t>Gourmandise de Noël</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Beschermengel</t>
+          <t>Kerstlekkernij</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -5579,48 +5579,161 @@
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Oolong — fraise, goji</t>
+          <t>Rooibos — amande, ananas</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>Oolong — aardbei, goji</t>
+          <t>Rooibos — amandel, ananas</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>22/02/2028</t>
-        </is>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="4" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="L46" s="5" t="n">
         <v>0.06</v>
       </c>
       <c r="M46" s="4" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/Gourmandise_de_noel.png?v=1769590512</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>https://teatower.com/products/rooibos-amande-gourmandise-de-noel-teatower</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Gourmandise de Noël – Rooibos Pâte d’Amande &amp; Ananas
+Laissez-vous séduire par Gourmandise de Noël, un rooibos festif mêlant la douceur de la pâte d’amande à la fraîcheur fruitée des morceaux d’ananas. Une infusion sans théine, idéale pour les instants cocooning de l’hiver.
+Recette &amp; préparation
+•
+Contenu : vrac 100 Gr
+•
+Dosage : 1–2 c. à café pour 250 ml
+•
+Température : 95 °C
+•
+Infusion : 7–10 minutes
+Ingrédients
+• Rooibos d’Afrique du Sud (69%)
+• Morceaux d’ananas (sucre de canne, ananas, acide citrique)
+• Arôme
+• Amandes hachées et effilées**
+• Sucre perlé
+**Ingrédient allergène : amandes.
+Astuce dégustation : savourez chaud, accompagné d’un biscuit de Noël, pour une pause douce et gourmande. 🎄</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>Kerstlekkernij – Rooibos Amandelspijs &amp; Ananas
+Laat je verleiden door Kerstlekkernij, een feestelijke rooibos die de zachtheid van amandelspijs vermengt met de fruitige frisheid van ananasstuktjes. Een infusie zonder cafeïne, ideaal voor warme winterse momenten vol gezelligheid.
+Recept &amp; bereiding
+•
+Inhoud: los 100 gr
+•
+Dosering: 1–2 theelepels voor 250 ml
+•
+Temperatuur: 95 °C
+•
+Trektijd: 7–10 minuten
+Ingrediënten
+• Rooibos uit Zuid-Afrika (69%)
+• Ananasstuktjes (rietsuiker, ananas, citroenzuur)
+• Aroma
+• Gehakte en gefileerde amandelen**
+• Parelsulker
+**Allergeen ingrediënt: amandelen.
+Proeftip: geniet warm, met een kerstkoekje erbij, voor een zachte en heerlijke pauze. 🎄</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>V0742</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>5413393800358</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Ange Gardien</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Beschermengel</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>100 g vrac</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Oolong — fraise, goji</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Oolong — aardbei, goji</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>22/02/2028</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L47" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M47" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N46" s="4" t="n">
+      <c r="N47" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O46" s="4" t="n">
+      <c r="O47" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P46" s="2" t="inlineStr">
+      <c r="P47" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0742-Ange-Gardien-Oolong-mangue-fraise-Ange-Gardien-Teatower.jpg?v=1762729392</t>
         </is>
       </c>
-      <c r="Q46" s="2" t="inlineStr">
+      <c r="Q47" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/oolong-mangue-fraise-ange-gardien-teatower</t>
         </is>
       </c>
-      <c r="R46" s="2" t="inlineStr">
+      <c r="R47" s="2" t="inlineStr">
         <is>
           <t>Ange Gardien
 Le thé oolong parfumé Ange Gardien marie délicatement Goji – Fraise pour une tasse fruitée, douce et réconfortante. Un oolong faible en théine, parfait pour une pause gourmande à tout moment de la journée.
@@ -5638,7 +5751,7 @@
 Moment de consommation : Au choix</t>
         </is>
       </c>
-      <c r="S46" s="2" t="inlineStr">
+      <c r="S47" s="2" t="inlineStr">
         <is>
           <t>Ange Gardien
 De geparfumeerde oolong thee Ange Gardien combineert delicaat Goji – Aardbei voor een fruitige, zachte en troostende kop thee. Een oolong arm aan cafeïne, perfect voor een lekkere pauze op elk moment van de dag.
@@ -5657,77 +5770,77 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>V0788</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>5413393800624</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Japan Sencha Yamato</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Japan Sencha Yamato</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>50g vrac</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="3" t="inlineStr">
         <is>
           <t>Thé vert nature — Sencha du Japon</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>Groene thee natuur — Japanse Sencha</t>
         </is>
       </c>
-      <c r="I47" s="2" t="n">
+      <c r="I48" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>01/04/2028</t>
         </is>
       </c>
-      <c r="K47" s="4" t="n">
+      <c r="K48" s="4" t="n">
         <v>18.5</v>
       </c>
-      <c r="L47" s="5" t="n">
+      <c r="L48" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M47" s="4" t="n">
+      <c r="M48" s="4" t="n">
         <v>17.45</v>
       </c>
-      <c r="N47" s="4" t="n">
+      <c r="N48" s="4" t="n">
         <v>11.1</v>
       </c>
-      <c r="O47" s="4" t="n">
+      <c r="O48" s="4" t="n">
         <v>10.47</v>
       </c>
-      <c r="P47" s="2" t="inlineStr">
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0788-Japan-Sencha-Yamato-Finest-quality-The-vert-nature-Japan-Sencha-Yamato-Teatower.jpg?v=1762729417</t>
         </is>
       </c>
-      <c r="Q47" s="2" t="inlineStr">
+      <c r="Q48" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/the-vert-nature-japan-sencha-yamato-teatower</t>
         </is>
       </c>
-      <c r="R47" s="2" t="inlineStr">
+      <c r="R48" s="2" t="inlineStr">
         <is>
           <t>Japan Sencha Yamato – Finest quality
 Le Japan Sencha Yamato – Finest quality est un thé vert d’exception, issu de feuilles de Sencha haut de gamme du Japon. Référence emblématique des thés verts japonais, il séduit par son caractère à la fois végétal, frais et intensément aromatique.
@@ -5745,7 +5858,7 @@
 Moment de consommation : Journée</t>
         </is>
       </c>
-      <c r="S47" s="2" t="inlineStr">
+      <c r="S48" s="2" t="inlineStr">
         <is>
           <t>Japan Sencha Yamato – Finest quality
 De Japan Sencha Yamato – Finest quality is een uitzonderlijke groene thee, afkomstig van premium Sencha bladeren uit Japan. Deze emblematische referentie van Japanse groene theeën bekoort door zijn karakter dat tegelijk vegetaal, fris en intens aromatisch is.
@@ -5764,77 +5877,77 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>V0793</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>5413393800341</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Orangipane</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Orangipane</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Thé vert — orange, amande, fleur d'oranger</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>Groene thee — sinaasappel, amandel, oranjebloesem</t>
         </is>
       </c>
-      <c r="I48" s="2" t="n">
+      <c r="I49" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>18/03/2028</t>
         </is>
       </c>
-      <c r="K48" s="4" t="n">
+      <c r="K49" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L48" s="5" t="n">
+      <c r="L49" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M48" s="4" t="n">
+      <c r="M49" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N48" s="4" t="n">
+      <c r="N49" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O48" s="4" t="n">
+      <c r="O49" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P48" s="2" t="inlineStr">
+      <c r="P49" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0793-Orangipane-The-vert-orange-amande-Orangipane-Teatower.jpg?v=1762729419</t>
         </is>
       </c>
-      <c r="Q48" s="2" t="inlineStr">
+      <c r="Q49" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/the-vert-orange-amande-orangipane-teatower</t>
         </is>
       </c>
-      <c r="R48" s="2" t="inlineStr">
+      <c r="R49" s="2" t="inlineStr">
         <is>
           <t>Orangipane
 L’Orangipane est un thé vert parfumé gourmand et chaleureux,
@@ -5860,7 +5973,7 @@
 Moment de consommation : Journée</t>
         </is>
       </c>
-      <c r="S48" s="2" t="inlineStr">
+      <c r="S49" s="2" t="inlineStr">
         <is>
           <t>Orangipane
 Orangipane is een geparfumeerde groene thee met een verwarmende, verwennende smaak,
@@ -5887,77 +6000,77 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>V0822</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>5413393808422</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Sous les cocotiers</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Sous les cocotiers</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>Infusion de fruits — coco, melon</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>Vruchteninfusie — kokos, meloen</t>
         </is>
       </c>
-      <c r="I49" s="2" t="n">
+      <c r="I50" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>11/02/2028</t>
         </is>
       </c>
-      <c r="K49" s="4" t="n">
+      <c r="K50" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L49" s="5" t="n">
+      <c r="L50" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M49" s="4" t="n">
+      <c r="M50" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N49" s="4" t="n">
+      <c r="N50" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O49" s="4" t="n">
+      <c r="O50" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P49" s="2" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0822-Sous-les-cocotiers-Infusion-de-fruits-coco-melon-Sous-les-cocotiers-Teatower.jpg?v=1762729457</t>
         </is>
       </c>
-      <c r="Q49" s="2" t="inlineStr">
+      <c r="Q50" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/infusion-de-fruits-coco-melon-sous-les-cocotiers-teatower</t>
         </is>
       </c>
-      <c r="R49" s="2" t="inlineStr">
+      <c r="R50" s="2" t="inlineStr">
         <is>
           <t>Sous les cocotiers
 Premier jour de vacances. Vous êtes allongé sur le sable chaud, une brise légère apporte un parfum de coco et de melon. Quelqu’un vous tend un verre fraîchement pressé. Vous fermez les yeux et souriez. Sous les cocotiers, c’est ce moment-là — en infusion.
@@ -5986,7 +6099,7 @@
 Le saviez-vous ? Le cocotier est appelé “l’arbre de vie” car chaque partie est utilisable : l’eau, le lait, la chair, l’huile, la coque (charbon), les feuilles (toitures), et même les fibres (cordage). Un seul cocotier peut produire pendant 80 ans. C’est la nature à son meilleur.</t>
         </is>
       </c>
-      <c r="S49" s="2" t="inlineStr">
+      <c r="S50" s="2" t="inlineStr">
         <is>
           <t>Onder de Kokospalmen
 Eerste vakantiedag. Je ligt languit op het warme zand, een lichte bries brengt de geur van kokos en meloen. Iemand reikt je een vers geperst glas aan. Je sluit je ogen en glimlacht. Onder de Kokospalmen, dat is dit moment — als infusie.
@@ -6016,77 +6129,77 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>V0838</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>5413393812023</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>framboise rose</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>framboos roos</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Oolong — framboise, rose</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>Oolong — framboos, roos</t>
         </is>
       </c>
-      <c r="I50" s="2" t="n">
+      <c r="I51" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>27/12/2027</t>
         </is>
       </c>
-      <c r="K50" s="4" t="n">
+      <c r="K51" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L50" s="5" t="n">
+      <c r="L51" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M50" s="4" t="n">
+      <c r="M51" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N50" s="4" t="n">
+      <c r="N51" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O50" s="4" t="n">
+      <c r="O51" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P50" s="2" t="inlineStr">
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0838-Oolong-Framboise-Oolong-Framboise-Teatower.jpg?v=1762729482</t>
         </is>
       </c>
-      <c r="Q50" s="2" t="inlineStr">
+      <c r="Q51" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/oolong-framboise-teatower</t>
         </is>
       </c>
-      <c r="R50" s="2" t="inlineStr">
+      <c r="R51" s="2" t="inlineStr">
         <is>
           <t>Oolong Framboise
 Oolong Framboise est un oolong parfumé délicatement fruité, associant la fraîcheur acidulée de la framboise à la douceur florale de la rose. Cette création élégante offre une tasse harmonieuse, à la fois gourmande et raffinée, idéale pour un moment de plaisir tout en légèreté.
@@ -6104,7 +6217,7 @@
 Moment de consommation : Au choix</t>
         </is>
       </c>
-      <c r="S50" s="2" t="inlineStr">
+      <c r="S51" s="2" t="inlineStr">
         <is>
           <t>Oolong Framboise
 Oolong Framboise is een geparfumeerde oolong vol delicate fruitigheid, die de frisse zuurheid van frambozen combineert met de bloemige zachtheid van roos. Deze elegante creatie biedt een harmonieuze kop, tegelijk smaakvol en verfijnd, ideaal voor een moment van puur genot in alle lichtheid.
@@ -6123,77 +6236,77 @@
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>V0847</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>5413393812269</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Pastèque Fraîcheur (ancien nom Couleur Mojito)</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Watermeloen Frisheid</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Infusion de fruits — pastèque, menthe, sureau</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>Vruchteninfusie — watermeloen, munt, vlierbes</t>
         </is>
       </c>
-      <c r="I51" s="2" t="n">
+      <c r="I52" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>01/03/2028</t>
         </is>
       </c>
-      <c r="K51" s="4" t="n">
+      <c r="K52" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L51" s="5" t="n">
+      <c r="L52" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M51" s="4" t="n">
+      <c r="M52" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N51" s="4" t="n">
+      <c r="N52" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O51" s="4" t="n">
+      <c r="O52" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P51" s="2" t="inlineStr">
+      <c r="P52" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0847-Couleur-Mojito-Infusion-de-fruits-pasteque-menthe-Couleur-Mojito-Teatower.jpg?v=1762729500</t>
         </is>
       </c>
-      <c r="Q51" s="2" t="inlineStr">
+      <c r="Q52" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/infusion-de-fruits-pasteque-menthe-couleur-mojito-teatower</t>
         </is>
       </c>
-      <c r="R51" s="2" t="inlineStr">
+      <c r="R52" s="2" t="inlineStr">
         <is>
           <t>Pastèque fraîcheur
 C'est l'heure de la sieste. Dehors, l'été pèse lourd. Vous ouvrez le frigo et sortez une pastèque bien fraîche — ce parfum sucré qui embaume la cuisine, ce bruit sourd du couteau qui tranche... Voilà exactement ce que cette infusion capture dans votre tasse. Une tranche d'été, à boire.
@@ -6212,7 +6325,7 @@
 Laissez refroidir quelques heures au frigo avec des glaçons — vous obtiendrez un thé glacé maison qui rivalise avec les plus belles limonades d'été.</t>
         </is>
       </c>
-      <c r="S51" s="2" t="inlineStr">
+      <c r="S52" s="2" t="inlineStr">
         <is>
           <t>```html
 Pastèque fraîcheur
@@ -6234,77 +6347,77 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>V0870</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>5413393813341</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>French Riviera</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>French Riviera</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Pu erh — églantier, maté, citron</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>Pu-erh — rozenbottel, maté, citroen</t>
         </is>
       </c>
-      <c r="I52" s="2" t="n">
+      <c r="I53" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>04/02/2028</t>
         </is>
       </c>
-      <c r="K52" s="4" t="n">
+      <c r="K53" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L52" s="5" t="n">
+      <c r="L53" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M52" s="4" t="n">
+      <c r="M53" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N52" s="4" t="n">
+      <c r="N53" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O52" s="4" t="n">
+      <c r="O53" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P52" s="2" t="inlineStr">
+      <c r="P53" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0870-French-Riviera-Pu-erh-citron-fruit-rouge-French-Riviera-Teatower.jpg?v=1762729534</t>
         </is>
       </c>
-      <c r="Q52" s="2" t="inlineStr">
+      <c r="Q53" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/pu-erh-citron-fruit-rouge-french-riviera-teatower</t>
         </is>
       </c>
-      <c r="R52" s="2" t="inlineStr">
+      <c r="R53" s="2" t="inlineStr">
         <is>
           <t>French Riviera
 Le French Riviera est un pu-erh parfumé aux notes fraîches et végétales d’églantier, de maté et de citron. Inspirée de l’art de vivre méditerranéen, cette création offre une tasse équilibrée, légèrement tonique et agréablement citronnée, idéale à tout moment de la journée.
@@ -6322,7 +6435,7 @@
 Moment de consommation : Au choix</t>
         </is>
       </c>
-      <c r="S52" s="2" t="inlineStr">
+      <c r="S53" s="2" t="inlineStr">
         <is>
           <t>French Riviera
 De French Riviera is een gearomatiseerde pu-erh met frisse en plantaardige tonen van rozenbottel, maté en citroen. Geïnspireerd door de mediterrane levensstijl, biedt deze creatie een gebalanceerd kopje, licht tonisch en aangenaam citroenzuur, ideaal op elk moment van de dag.
@@ -6341,77 +6454,77 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>V0875</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>5413393813136</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Evasion Ambrée</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Evasion Ambrée</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Rooibos — orange, cassis, cannelle</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>Rooibos — sinaasappel, zwarte bes, kaneel</t>
         </is>
       </c>
-      <c r="I53" s="2" t="n">
+      <c r="I54" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>12/12/2027</t>
         </is>
       </c>
-      <c r="K53" s="4" t="n">
+      <c r="K54" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L53" s="5" t="n">
+      <c r="L54" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M53" s="4" t="n">
+      <c r="M54" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N53" s="4" t="n">
+      <c r="N54" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O53" s="4" t="n">
+      <c r="O54" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P53" s="2" t="inlineStr">
+      <c r="P54" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0875-Souvenir-de-La-havane-Rooibos-rhum-Souvenir-de-La-Havane-Teatower.jpg?v=1762729544</t>
         </is>
       </c>
-      <c r="Q53" s="2" t="inlineStr">
+      <c r="Q54" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/rooibos-rhum-souvenir-de-la-havane-teatower</t>
         </is>
       </c>
-      <c r="R53" s="2" t="inlineStr">
+      <c r="R54" s="2" t="inlineStr">
         <is>
           <t>Evasion ambrée
 Évasion Ambrée, la nouvelle identité de notre rooibos Souvenir de la Havane. Sans changer sa recette, ce nouveau nom met parfaitement en avant son univers chaleureux, épicé et délicatement fruité, inspiré des ambiances solaires et ambrées.
@@ -6430,7 +6543,7 @@
 Moment de consommation : Au choix</t>
         </is>
       </c>
-      <c r="S53" s="2" t="inlineStr">
+      <c r="S54" s="2" t="inlineStr">
         <is>
           <t>Evasion ambrée
 Évasion Ambrée, de nieuwe identiteit van onze rooibos Souvenir de la Havane. Zonder de receptuur te wijzigen, brengt deze nieuwe naam perfect zijn warme, gekruide en delicaat fruitige universum naar voren, geïnspireerd door zonrijke en amberen sferen.
@@ -6450,77 +6563,77 @@
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>V0885</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>5413393814133</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Cococabana</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Cococabana</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Thé vert — coco, ananas</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Groene thee — kokos, ananas</t>
         </is>
       </c>
-      <c r="I54" s="2" t="n">
+      <c r="I55" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t>22/02/2028</t>
         </is>
       </c>
-      <c r="K54" s="4" t="n">
+      <c r="K55" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L54" s="5" t="n">
+      <c r="L55" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M54" s="4" t="n">
+      <c r="M55" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N54" s="4" t="n">
+      <c r="N55" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O54" s="4" t="n">
+      <c r="O55" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P54" s="2" t="inlineStr">
+      <c r="P55" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0885-Cococabana-The-vert-coco-Cococabana-Teatower.jpg?v=1762729561</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="inlineStr">
+      <c r="Q55" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/the-vert-coco-cococabana-teatower</t>
         </is>
       </c>
-      <c r="R54" s="2" t="inlineStr">
+      <c r="R55" s="2" t="inlineStr">
         <is>
           <t>Cococabana
 Cococabana est un thé vert parfumé exotique et ensoleillé, qui marie la fraîcheur végétale du thé vert Sencha à la douceur gourmande de la noix de coco et aux notes fruitées de l’ananas. Une invitation à l’évasion, idéale pour une pause dépaysante.
@@ -6538,7 +6651,7 @@
 Moment de consommation : Journée</t>
         </is>
       </c>
-      <c r="S54" s="2" t="inlineStr">
+      <c r="S55" s="2" t="inlineStr">
         <is>
           <t>Cococabana
 Cococabana is een exotische en zonnige gearomatiseerde groene thee, die de plantaardige frisheid van Sencha groene thee combineert met de verwennende zoetheid van kokos en de fruitige toetsen van ananas. Een uitnodiging tot ontsnapping, ideaal voor een ontspannende pauze vol exotiek.
@@ -6557,77 +6670,77 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>V0889</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>5413393814218</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Granada</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Maté — grenade, citron</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>Maté — granaatappel, citroen</t>
         </is>
       </c>
-      <c r="I55" s="2" t="n">
+      <c r="I56" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>04/01/2028</t>
         </is>
       </c>
-      <c r="K55" s="4" t="n">
+      <c r="K56" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L55" s="5" t="n">
+      <c r="L56" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M55" s="4" t="n">
+      <c r="M56" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N55" s="4" t="n">
+      <c r="N56" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O55" s="4" t="n">
+      <c r="O56" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P55" s="2" t="inlineStr">
+      <c r="P56" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0889-Granada-Mate-grenade-Granada-Teatower.jpg?v=1762729571</t>
         </is>
       </c>
-      <c r="Q55" s="2" t="inlineStr">
+      <c r="Q56" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/mate-grenade-granada-teatower</t>
         </is>
       </c>
-      <c r="R55" s="2" t="inlineStr">
+      <c r="R56" s="2" t="inlineStr">
         <is>
           <t>Granada
 Granada est un maté parfumé aux notes fraîches et acidulées de grenade et de citron. Tonique et fruité, ce mélange offre une infusion vivifiante et équilibrée, idéale pour stimuler l’énergie et accompagner les débuts de journée.
@@ -6645,7 +6758,7 @@
 Moment de consommation : Matin</t>
         </is>
       </c>
-      <c r="S55" s="2" t="inlineStr">
+      <c r="S56" s="2" t="inlineStr">
         <is>
           <t>Granada
 Granada is een gearomatiseerde maté met frisse en pittige noten van granaatappel en citroen. Verkwikkend en fruitig, deze blend biedt een stimulerende en evenwichtige infusie, ideaal om de energie aan te wakkeren en de ochtendrituelen te begeleiden.
@@ -6664,77 +6777,184 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>V0891</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>5413393814867</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Trésor des lutins</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Schat van de elfen</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>100 g vrac</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Infusion de fruits — chocolat, noisette</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Vruchteninfusie — chocolade, hazelnoot</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L57" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M57" s="4" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="N57" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="O57" s="4" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/Tresor_des_lutins.png?v=1769592963</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>https://teatower.com/products/infusion-de-fruits-chocolat-noisette-tresor-des-lutins-teatower</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Trésor des Lutins
+Au fond de l'atelier du Père Noël, derrière les piles de cadeaux, les lutins cachent un secret : une recette de fruits d'hiver, de cacao et de noisette grillée qu'ils sirotent en riant quand personne ne regarde. C'est cette recette que nous avons volée pour vous. Le Trésor des Lutins, c'est Noël en une gorgée — gourmand, réconfortant, et naturellement sans théine.
+Les éclats de cacao et les feuilles d'amandier apportent une profondeur chocolatée, tandis que les pétales de rose et les fleurs de carthame ajoutent une touche de couleur et de délicatesse. La tasse est ambrée, le parfum envoûtant, et chaque gorgée rappelle les bonbons de Noël qu'on volait dans le sapin.
+Recette &amp; préparation
+•
+Contenu : 100 g en vrac
+•
+Dosage : 1 à 2 c. à café pour 250 ml
+•
+Température : 95 °C
+•
+Infusion : 8 à 10 minutes — laissez le temps aux arômes de se libérer
+Ingrédients
+Morceaux de pomme (pomme, acide citrique), écorces et brisures de cacao, feuilles d'amandier, pétales de rose rouge, bleuet blanc, fleurs de carthame, arôme naturel.
+Allergène : amandes.
+Astuce : ajoutez une pointe de lait végétal pour un effet chocolat chaud d'hiver — les enfants adorent.</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>Trésor des Lutins
+Diep in de werkplaats van de Kerstman, achter de stapels cadeaus, verbergen de kabouters een geheim: een recept van wintervruchten, cacao en geroosterde hazelnoot dat ze lachend nippen wanneer niemand kijkt. Dit recept hebben we voor u gestolen. De Trésor des Lutins, dat is Kerstmis in één teug — verwennend, troostend, en natuurlijk zonder cafeïne.
+De cacaoschilfers en amandelbladeren brengen een chocoladeachtige diepte, terwijl de rozenblaadjes en saffloerbloemen een vleugje kleur en finesse toevoegen. De kop is amber, het aroma betoverend, en elke teug herinnert aan de kerstbonbons die we stiekem uit de boom pikten.
+Recept &amp; bereiding
+•
+Inhoud: 100 g los
+•
+Dosering: 1 tot 2 theelepels voor 250 ml
+•
+Temperatuur: 95 °C
+•
+Infusie: 8 tot 10 minuten — geef de aroma's de tijd om vrij te komen
+Ingrediënten
+Appelstukjes (appel, citroenzuur), cacaoschillen en -brokken, amandelbladeren, rode rozenblaadjes, witte korenbloem, saffloerbloemen, natuurlijk aroma.
+Allergeen: amandelen.
+Tip: voeg een scheutje plantaardige melk toe voor een warme chocolademelk-effect — kinderen zijn er dol op.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>V0899</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>5413393815062</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Festival Fruité (ancien nom Mumbai Mango) BIO</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Festival Fruité (vroeger Mumbai Mango) BIO</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Infusion de fruits BIO — pomme, orange, fraise, mangue</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>Vruchteninfusie BIO — appel, sinaasappel, aardbei, mango</t>
         </is>
       </c>
-      <c r="I56" s="2" t="n">
+      <c r="I58" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
         <is>
           <t>24/08/2027</t>
         </is>
       </c>
-      <c r="K56" s="4" t="n">
+      <c r="K58" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L56" s="5" t="n">
+      <c r="L58" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M56" s="4" t="n">
+      <c r="M58" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N56" s="4" t="n">
+      <c r="N58" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O56" s="4" t="n">
+      <c r="O58" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P56" s="2" t="inlineStr">
+      <c r="P58" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0899-Mumbai-Mango-BIO-Infusion-de-fruits-mangue-Mumbai-Mango-BIO-Teatower.jpg?v=1762729586</t>
         </is>
       </c>
-      <c r="Q56" s="2" t="inlineStr">
+      <c r="Q58" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/infusion-de-fruits-mangue-mumbai-mango-bio-teatower</t>
         </is>
       </c>
-      <c r="R56" s="2" t="inlineStr">
+      <c r="R58" s="2" t="inlineStr">
         <is>
           <t>Festival Fruité
 C'est dimanche matin, la cuisine sent bon les crêpes. Sur la table, les pots de confiture s'alignent comme des promesses colorées — fraise de Wépion, orange amère, compote de pommes du verger. Vous respirez cette symphonie fruitée et souriez. Dans votre tasse, Festival Fruité raconte exactement cette histoire : l'innocence des matins sucrés, la générosité des fruits qui s'entremêlent.
@@ -6754,7 +6974,7 @@
 Astuce : Préparez-la glacée avec une rondelle d'orange fraîche — vos invités penseront à un cocktail sans alcool sophistiqué.</t>
         </is>
       </c>
-      <c r="S56" s="2" t="inlineStr">
+      <c r="S58" s="2" t="inlineStr">
         <is>
           <t>Festival Fruité
 Het is zondagochtend, de keuken ruikt naar versgebakken pannenkoeken. Op tafel staan de jampotten op een rij als kleurrijke beloftes — Wépion-aardbeien, bittere sinaasappel, appelcompote uit de boomgaard. Je ademt deze fruitige symfonie in en glimlacht. In je kopje vertelt Festival Fruité precies dit verhaal: de onschuld van zoete ochtenden, de vrijgevigheid van vruchten die elkaar omarmen.
@@ -6775,77 +6995,77 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>V0900</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>5413393815093</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Bora Bora BIO</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Bora Bora BIO</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Thé noir BIO — pêche, ananas, citronnelle</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>Zwarte thee BIO — perzik, ananas, citroengras</t>
         </is>
       </c>
-      <c r="I57" s="2" t="n">
+      <c r="I59" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
         <is>
           <t>13/08/2027</t>
         </is>
       </c>
-      <c r="K57" s="4" t="n">
+      <c r="K59" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="L57" s="5" t="n">
+      <c r="L59" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M57" s="4" t="n">
+      <c r="M59" s="4" t="n">
         <v>9.91</v>
       </c>
-      <c r="N57" s="4" t="n">
+      <c r="N59" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="O57" s="4" t="n">
+      <c r="O59" s="4" t="n">
         <v>5.94</v>
       </c>
-      <c r="P57" s="2" t="inlineStr">
+      <c r="P59" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/0900-Bora-Bora-BIO-The-noir-aromatise-passion-Bora-Bora-BIO-Teatower_4f2e9195-322a-4284-a012-885b550ea23f.jpg?v=1762729589</t>
         </is>
       </c>
-      <c r="Q57" s="2" t="inlineStr">
+      <c r="Q59" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/the-noir-aromatise-passion-bora-bora-bio-teatower</t>
         </is>
       </c>
-      <c r="R57" s="2" t="inlineStr">
+      <c r="R59" s="2" t="inlineStr">
         <is>
           <t>Bora Bora - BIO
 Bora Bora - BIO est un thé noir parfumé biologique aux saveurs exotiques et ensoleillées de pêche, de citronnelle et d’ananas. Évocateur d’évasion et de douceur tropicale, il offre une infusion fruitée et rafraîchissante, idéale pour une dégustation en journée.
@@ -6866,7 +7086,7 @@
 Moment de consommation : Journée</t>
         </is>
       </c>
-      <c r="S57" s="2" t="inlineStr">
+      <c r="S59" s="2" t="inlineStr">
         <is>
           <t>Bora Bora - BIO
 Bora Bora - BIO is een biologische gearomatiseerde zwarte thee met exotische en zonnige smaken van perzik, citroengras en ananas. Deze thee roept beelden op van ontsnapping en tropische zachtheid en biedt een fruitige en verfrissende infusie, ideaal voor overdag.
@@ -6888,73 +7108,73 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>V0905</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>5413393807913</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Un Noël Vanillé</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Een Gevanielleerde Kerst</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>100 g vrac</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Oolong, thé blanc &amp; vert — vanille, amande, pomme</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>Oolong, witte &amp; groene thee — vanille, amandel, appel</t>
         </is>
       </c>
-      <c r="I58" s="2" t="n">
+      <c r="I60" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="J58" s="2" t="inlineStr"/>
-      <c r="K58" s="4" t="n">
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L58" s="5" t="n">
+      <c r="L60" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M58" s="4" t="n">
+      <c r="M60" s="4" t="n">
         <v>11.32</v>
       </c>
-      <c r="N58" s="4" t="n">
+      <c r="N60" s="4" t="n">
         <v>7.2</v>
       </c>
-      <c r="O58" s="4" t="n">
+      <c r="O60" s="4" t="n">
         <v>6.79</v>
       </c>
-      <c r="P58" s="2" t="inlineStr">
+      <c r="P60" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/Un_noel_vanille.png?v=1769590364</t>
         </is>
       </c>
-      <c r="Q58" s="2" t="inlineStr">
+      <c r="Q60" s="2" t="inlineStr">
         <is>
           <t>https://teatower.com/products/un-noel-vanille-oolong-parfume-vanille-teatower</t>
         </is>
       </c>
-      <c r="R58" s="2" t="inlineStr">
+      <c r="R60" s="2" t="inlineStr">
         <is>
           <t>Un Noël Vanillé – Thé Oolong, Blanc &amp; Vert aux Saveurs de Fêtes
 Découvrez Un Noël Vanillé, une infusion raffinée et festive qui marie la douceur de la pomme, la chaleur de la cannelle et la gourmandise de la vanille. Élaborée sur une base de Oolong, de thé blanc et de thé vert, cette création Teatower offre une tasse élégante et délicatement parfumée, parfaite pour les instants cocooning de l’hiver.
@@ -6978,7 +7198,7 @@
 Astuce dégustation : savourez ce thé chaud pour accompagner un dessert de fête, ou froid pour une pause vanillée rafraîchissante. 🎄🍏</t>
         </is>
       </c>
-      <c r="S58" s="2" t="inlineStr">
+      <c r="S60" s="2" t="inlineStr">
         <is>
           <t>Un Noël Vanillé – Oolong, Witte &amp; Groene Thee met Feestelijke Smaken
 Ontdek Un Noël Vanillé, een verfijnde en feestelijke infusie die de zoetheid van appel, de warmte van kaneel en de verleidelijke smaak van vanille samenbrengt. Gebaseerd op een blend van Oolong, witte thee en groene thee, biedt deze Teatower-creatie een elegante en delicaat geparfumeerde kop thee, perfect voor knusse wintermomenten.
@@ -7003,69 +7223,180 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>V0913</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>5413393003902</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Féérie d'Hiver</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Wintersprookje</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>100 g vrac</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Infusion de fruits — canneberge, orange</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Vruchteninfusie — veenbes, sinaasappel</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L61" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M61" s="4" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="N61" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="O61" s="4" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003902-Feerie-dHiver.jpg?v=1762730488</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr"/>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Féérie d’Hiver – Infusion Canneberge &amp; Orange
+Plongez dans Féérie d’Hiver, une infusion fruitée et envoûtante qui marie la douceur des canneberges à la fraîcheur de l’orange et à l’intensité des baies d’hiver. Une boisson festive et sans théine, idéale pour vos instants cocooning durant la saison froide.
+Recette &amp; préparation
+•
+Contenu : vrac 100 Gr
+•
+Dosage : 1–2 c. à café pour 250 ml
+•
+Température : 95 °C
+•
+Infusion : 8–10 minutes
+Ingrédients
+• Grains de raisin huilés (raisins, huile de tournesol)
+• Canneberges entières et sucrées (canneberges, sucre, huile de tournesol)
+• Cristaux de sucre (sucre, farine de riz, matières grasses végétales (colza), fécule de pomme de terre, colorants : E120, E160a, arôme)
+• Baies de sorbier
+• Baies d’argousier
+• Fleurs de bleuet
+• Arôme
+Astuce dégustation : dégustez cette infusion bien chaude pour une pause fruitée et lumineuse, ou ajoutez-en quelques cuillères pour parfumer un vin chaud maison aux notes d’orange et de canneberge. 🍊🍷❄️</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>Wintersprookje – Cranberry &amp; Oranje Infusie (SEO-geoptimaliseerd)
+Dompel jezelf onder in Wintersprookje, een fruitige en betoverende infusie die de zoetheid van cranberries combineert met de frisheid van sinaasappel en de intensiteit van winterbessen. Een feestelijke en theïnevrije drank, ideaal voor jouw cocooning momenten tijdens het koude seizoen.
+Recept &amp; bereiding
+•
+Inhoud: losse thee 100 Gr
+•
+Dosering: 1–2 tl voor 250 ml
+•
+Temperatuur: 95 °C
+•
+Infusie: 8–10 minuten
+Ingrediënten
+• Geoliede rozijnen (rozijnen, zonnebloemolie)
+• Hele en gezoete cranberries (cranberries, suiker, zonnebloemolie)
+• Suikerkristallen (suiker, rijstmeel, plantaardige vetten (koolzaad), aardappelzetmeel, kleurstoffen: E120, E160a, aroma)
+• Lijsterbessen
+• Duindoornbessen
+• Korenbloembloemen
+• Aroma
+Degustatietip: geniet van deze infusie lekker warm voor een fruitige en heldere pauze, of voeg een paar lepels toe om een zelfgemaakte glühwein te parfumeren met tonen van sinaasappel en cranberry. 🍊🍷❄️</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>C0185</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>5413393003858</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>La petite boîte à infusions</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Het kleine infusiedoosje</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>Boîte 10 infusettes</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n"/>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>Coffret 10 infusettes sans théine : vanille-cannelle, cerise-amaretto, menthe-rose-lavande, masala chai, canneberge-orange</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>Doosje 10 theezakjes cafeïnevrij: vanille-kaneel, kers-amaretto, munt-roos-lavendel, masala chai, veenbes-sinaasappel</t>
         </is>
       </c>
-      <c r="I59" s="2" t="n">
+      <c r="I62" s="2" t="n">
         <v>171</v>
       </c>
-      <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="4" t="n">
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L59" s="5" t="n">
+      <c r="L62" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M59" s="4" t="n">
+      <c r="M62" s="4" t="n">
         <v>9.43</v>
       </c>
-      <c r="N59" s="4" t="n">
+      <c r="N62" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O59" s="4" t="n">
+      <c r="O62" s="4" t="n">
         <v>5.66</v>
       </c>
-      <c r="P59" s="2" t="inlineStr">
+      <c r="P62" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003858-La-petite-boite-a-infusions.jpg?v=1762730478</t>
         </is>
       </c>
-      <c r="Q59" s="2" t="inlineStr"/>
-      <c r="R59" s="2" t="inlineStr">
+      <c r="Q62" s="2" t="inlineStr"/>
+      <c r="R62" s="2" t="inlineStr">
         <is>
           <t>La Petite Boîte à Infusions — 10 Infusettes
 Petite par la taille, grande par les saveurs. Cette boîte tient dans la paume de la main, mais elle contient cinq voyages : les épices chaudes de l'Inde, la douceur de la Méditerranée, les nuits étoilées d'hiver, les cerises de Venise et le calme d'un jardin de roses. 10 infusettes, 5 univers, zéro théine.
@@ -7078,7 +7409,7 @@
 Le petit cadeau qui fait mouche. Format poche, prix doux, effet garanti. À glisser dans une carte, un sac ou sous le sapin.</t>
         </is>
       </c>
-      <c r="S59" s="2" t="inlineStr">
+      <c r="S62" s="2" t="inlineStr">
         <is>
           <t>Het Kleine Infusiedoosje — 10 Theezakjes
 Klein van formaat, groot van smaak. Dit doosje past in je handpalm, maar bevat vijf reizen: de warme kruiden van India, de zachtheid van de Middellandse Zee, de sterrenvolle winternachten, de kersen van Venetië en de rust van een rozentuin. 10 theezakjes, 5 werelden, geen cafeïne.
@@ -7092,69 +7423,69 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>C0186</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>5413393003841</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>La petite boîte à thés</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Het kleine theedoosje</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>Boîte 10 infusettes</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Coffret 10 infusettes de thé : spéculoos, cerise-jasmin, oolong vanille, orange-amande, pomme-cannelle</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>Doosje 10 theezakjes thee: speculaas, kers-jasmijn, oolong vanille, sinaasappel-amandel, appel-kaneel</t>
         </is>
       </c>
-      <c r="I60" s="2" t="n">
+      <c r="I63" s="2" t="n">
         <v>298</v>
       </c>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="4" t="n">
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L60" s="5" t="n">
+      <c r="L63" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M60" s="4" t="n">
+      <c r="M63" s="4" t="n">
         <v>9.43</v>
       </c>
-      <c r="N60" s="4" t="n">
+      <c r="N63" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O60" s="4" t="n">
+      <c r="O63" s="4" t="n">
         <v>5.66</v>
       </c>
-      <c r="P60" s="2" t="inlineStr">
+      <c r="P63" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003841-Coffret-cacahuete-The-2025.jpg?v=1762730481</t>
         </is>
       </c>
-      <c r="Q60" s="2" t="inlineStr"/>
-      <c r="R60" s="2" t="inlineStr">
+      <c r="Q63" s="2" t="inlineStr"/>
+      <c r="R63" s="2" t="inlineStr">
         <is>
           <t>La Petite Boîte à Thés — 10 Infusettes
 Pour ceux qui préfèrent la profondeur du thé à la légèreté de l'infusion. Cette petite boîte réunit cinq thés d'exception — du spéculoos belge à la pâtisserie orientale, en passant par la vanille de Noël et la pomme-cannelle de mamie. 10 sachets, 5 caractères, une seule certitude : vous allez trouver votre favori.
@@ -7167,7 +7498,7 @@
 Un petit prix, un grand effet. À offrir sans raison particulière — ou parce que les meilleurs cadeaux sont ceux qu'on n'attend pas.</t>
         </is>
       </c>
-      <c r="S60" s="2" t="inlineStr">
+      <c r="S63" s="2" t="inlineStr">
         <is>
           <t>De Kleine Theedoos — 10 Theezakjes
 Voor wie de diepte van thee verkiest boven de lichtheid van tisanes. Deze kleine doos verenigt vijf uitzonderlijke theeën — van Belgische speculoos tot oosterse patisserie, via kerstvanille en oma's appel-kaneel. 10 zakjes, 5 karakters, één zekerheid: u gaat uw favoriet vinden.
@@ -7181,69 +7512,69 @@
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>C0187</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>5413393003865</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Coffret découverte de Noël</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Kerst ontdekkingsbox</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>Coffret 25 infusettes</t>
         </is>
       </c>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Coffret 25 infusettes : cacao-noisette, rooibos amande, orange-cannelle, oolong vanille, canneberge-orange</t>
         </is>
       </c>
-      <c r="H61" s="3" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>Box 25 theezakjes: cacao-hazelnoot, rooibos amandel, sinaasappel-kaneel, oolong vanille, veenbes-sinaasappel</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n">
+      <c r="I64" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="4" t="n">
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L61" s="5" t="n">
+      <c r="L64" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M61" s="4" t="n">
+      <c r="M64" s="4" t="n">
         <v>14.15</v>
       </c>
-      <c r="N61" s="4" t="n">
+      <c r="N64" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O61" s="4" t="n">
+      <c r="O64" s="4" t="n">
         <v>8.49</v>
       </c>
-      <c r="P61" s="2" t="inlineStr">
+      <c r="P64" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003865-Coffret-decouverte-de-Noel-2025.jpg?v=1762730484</t>
         </is>
       </c>
-      <c r="Q61" s="2" t="inlineStr"/>
-      <c r="R61" s="2" t="inlineStr">
+      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="R64" s="2" t="inlineStr">
         <is>
           <t>Coffret Découverte de Noël — 25 Infusettes Festives
 Imaginez : dehors, le froid de décembre. Dedans, vos mains enveloppent une tasse fumante aux parfums de cannelle, de cacao et d'orange confite. Le Coffret Découverte de Noël, c'est ce moment-là — multiplié par 25. Cinq créations Teatower réunies dans un seul coffret, pour transformer chaque matin de décembre en petit rituel gourmand.
@@ -7260,7 +7591,7 @@
 Pour qui ? Pour la personne qui vous dit toujours "rien, merci" quand vous demandez ce qui lui ferait plaisir. Ce coffret, c'est la réponse parfaite.</t>
         </is>
       </c>
-      <c r="S61" s="2" t="inlineStr">
+      <c r="S64" s="2" t="inlineStr">
         <is>
           <t>\
 \Kerst Ontdekkingsdoos – 25 Feestelijke Infusettes\
@@ -7297,69 +7628,69 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>C0188</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>5413393003872</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>La hotte de Noël</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>De kerstsok</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>Coffret 4 × 50 g + pince</t>
         </is>
       </c>
-      <c r="F62" s="2" t="n"/>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Coffret 4 × 50 g vrac + pince à thé : cacao-noisette, orange-cannelle, rooibos amande, canneberge-orange</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>Box 4 × 50 g losse thee + theeklem: cacao-hazelnoot, sinaasappel-kaneel, rooibos amandel, veenbes-sinaasappel</t>
         </is>
       </c>
-      <c r="I62" s="2" t="n">
+      <c r="I65" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="4" t="n">
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="L62" s="5" t="n">
+      <c r="L65" s="5" t="n">
         <v>0.06</v>
       </c>
-      <c r="M62" s="4" t="n">
+      <c r="M65" s="4" t="n">
         <v>37.74</v>
       </c>
-      <c r="N62" s="4" t="n">
+      <c r="N65" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="O62" s="4" t="n">
+      <c r="O65" s="4" t="n">
         <v>22.64</v>
       </c>
-      <c r="P62" s="2" t="inlineStr">
+      <c r="P65" s="2" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003872-La-hotte-de-Noel.jpg?v=1762730486</t>
         </is>
       </c>
-      <c r="Q62" s="2" t="inlineStr"/>
-      <c r="R62" s="2" t="inlineStr">
+      <c r="Q65" s="2" t="inlineStr"/>
+      <c r="R65" s="2" t="inlineStr">
         <is>
           <t>La Hotte de Noël — Coffret 4 Infusions en Vrac + Pince à Thé
 200 grammes de pur bonheur hivernal. Ouvrez la hotte et laissez les parfums vous envahir : le cacao grillé du Trésor des Lutins, les épices chaudes de l'Offrande des Rois Mages, l'amande douce de la Gourmandise de Noël, et la canneberge pétillante de la Féérie d'Hiver. Quatre boîtes, une pince à thé, des semaines de plaisir.
@@ -7374,7 +7705,7 @@
 Pour les amoureux du vrai thé. Ce coffret est fait pour ceux qui prennent le temps d'infuser, de sentir, de savourer.</t>
         </is>
       </c>
-      <c r="S62" s="2" t="inlineStr">
+      <c r="S65" s="2" t="inlineStr">
         <is>
           <t>De Kerstzak — Geschenkset 4 Losse Infusies + Theeklem
 200 gram puur wintergeluk. Open de zak en laat de geuren je overweldigen: de geroosterde cacao van Schat der Kaboutertjes, de warme kruiden van Geschenk der Wijzen, de zoete amandel van Kerstlekkernij, en de sprankelende cranberry van Wintersprookje. Vier doosjes, één theeklem, weken vol genot.
@@ -7390,340 +7721,6 @@
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>C0191</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>5413393004350</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Trésor des lutins</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Schat van de elfen</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Boîte 50 g</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="n"/>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>Infusion de fruits — chocolat, noisette</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>Vruchteninfusie — chocolade, hazelnoot</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L63" s="5" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M63" s="4" t="n">
-        <v>9.43</v>
-      </c>
-      <c r="N63" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O63" s="4" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="P63" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003872_3.png?v=1768229545</t>
-        </is>
-      </c>
-      <c r="Q63" s="2" t="inlineStr"/>
-      <c r="R63" s="2" t="inlineStr">
-        <is>
-          <t>Trésor des Lutins
-Au fond de l'atelier du Père Noël, les lutins cachent un secret. Quand les rires s'estompent et que l'ouvrage avance, ils s'accordent une pause autour d'un bol fumant qui sent la noisette grillée et le cacao. C'est leur trésor, celui qui réchauffe les cœurs avant la grande distribution. Une recette transmise de lutin en lutin, pour les moments où l'on a besoin de croire encore un peu à la magie.
-Dans votre tasse, cette infusion révèle une robe ambrée aux reflets cuivrés. La noisette grillée enveloppe le palais de sa douceur toastée, tandis que le cacao apporte une note chocolatée réconfortante. Les morceaux de pomme acidulés équilibrent cette gourmandise d'hiver, créant une harmonie parfaite entre fruité et torréfié.
-Ingrédients
-• Morceaux de pomme (pomme, acide citrique)
-• Écorces et brisures de cacao
-• Feuilles d'amandier
-• Pétales de rose rouge, bleuet blanc, fleurs de carthame
-• Arôme naturel
-**Ingrédient allergène : amandes.
-Conseils de préparation
-•
-Dosage : 1–2 c. à café pour 250 ml
-•
-Température : 95 °C
-•
-Infusion : 8–10 minutes
-•
-Théine : Sans théine
-•
-Moment idéal : Tout moment de la journée
-Astuce gourmande : Ajoutez une pointe de lait d'amande pour intensifier la note noisette de cette infusion de Noël.</t>
-        </is>
-      </c>
-      <c r="S63" s="2" t="inlineStr">
-        <is>
-          <t>Schatt van de Elfen – Kerstinfusie Hazelnoot &amp; Cacao (Theïne Vrij)
-Stap binnen in de betoverende werkplaats van de Kerstman: Schatt van de Elfen combineert de zachtheid van geroosterde hazelnoot met cacao en winterfruit, voor een heerlijke en natuurlijk theïnevrije kerstinfusie.
-Recept &amp; bereiding
-• Inhoud: los 50 Gr
-• Dosering: 1–2 tl voor 250 ml
-• Temperatuur: 95 °C
-• Infusie: 8–10 minuten
-Ingrediënten
-• Stukjes appel (appel, citroenzuur)
-• Cacaoschillen en -gruis
-• Amandelbladeren
-• Rode rozenblaadjes, witte korenbloem, saffloerbloemen
-• Natuurlijk aroma
-**Allergeen ingrediënt: amandelen.
-Tip voor proeven: ideaal op elk moment van de dag voor een zachte en gastronomische pauze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>C0192</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>5413393004367</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Gourmandise de Noël</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Kerstlekkernij</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Boîte 50 g</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n"/>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Rooibos — amande, ananas</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>Rooibos — amandel, ananas</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L64" s="5" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M64" s="4" t="n">
-        <v>9.43</v>
-      </c>
-      <c r="N64" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O64" s="4" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="P64" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003872_4.png?v=1768230036</t>
-        </is>
-      </c>
-      <c r="Q64" s="2" t="inlineStr">
-        <is>
-          <t>https://teatower.com/products/rooibos-amande-gourmandise-de-noel-teatower-1</t>
-        </is>
-      </c>
-      <c r="R64" s="2" t="inlineStr">
-        <is>
-          <t>Gourmandise de Noël – Rooibos Pâte d’Amande &amp; Ananas
-Laissez-vous séduire par Gourmandise de Noël, un rooibos festif mêlant la douceur de la pâte d’amande à la fraîcheur fruitée des morceaux d’ananas. Une infusion sans théine, idéale pour les instants cocooning de l’hiver.
-Recette &amp; préparation
-•
-Contenu : vrac 50 Gr
-•
-Dosage : 1–2 c. à café pour 250 ml
-•
-Température : 95 °C
-•
-Infusion : 7–10 minutes
-Ingrédients
-• Rooibos d’Afrique du Sud (69%)
-• Morceaux d’ananas (sucre de canne, ananas, acide citrique)
-• Arôme
-• Amandes hachées et effilées**
-• Sucre perlé
-**Ingrédient allergène : amandes.
-Astuce dégustation : savourez chaud, accompagné d’un biscuit de Noël, pour une pause douce et gourmande. 🎄</t>
-        </is>
-      </c>
-      <c r="S64" s="2" t="inlineStr">
-        <is>
-          <t>Kerstlekkernij – Rooibos Amandelpasta &amp; Ananas
-Laat u verleiden door Kerstlekkernij, een feestelijke rooibos die de zoetheid van amandelpasta combineert met de fruitige frisheid van ananasstukjes. Een cafeïnevrije infusie, ideaal voor knusse wintermomenten.
-Bereiding
-• Inhoud: 50 gr losse thee
-• Dosering: 1–2 theelepels per 250 ml
-• Temperatuur: 95°C
-• Trektijd: 7–10 minuten
-Ingrediënten
-• Rooibos uit Zuid-Afrika (69%)
-• Ananasstukjes (rietsuiker, ananas, citroenzuur)
-• Aroma
-• Gehakte en gesneden amandelen**
-• Parelsuiker
-**Allergeen: amandelen.
-Degustatietip: geniet warm, samen met een kerstkoekje, voor een zachte en heerlijke pauze. 🎄</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>C0193</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>5413393004374</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Féérie d'Hiver</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>Wintersprookje</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Boîte 50 g</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="n"/>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>Infusion de fruits — canneberge, orange</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>Vruchteninfusie — veenbes, sinaasappel</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L65" s="5" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M65" s="4" t="n">
-        <v>9.43</v>
-      </c>
-      <c r="N65" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O65" s="4" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="P65" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0761/7586/8243/files/5413393003872_5.png?v=1768229198</t>
-        </is>
-      </c>
-      <c r="Q65" s="2" t="inlineStr"/>
-      <c r="R65" s="2" t="inlineStr">
-        <is>
-          <t>Féérie d'Hiver
-Il neige dehors, et dans votre cuisine flotte déjà ce parfum de fête. Vous versez l'eau frémissante sur les canneberges écarlates et les écorces d'orange. Cinq minutes plus tard, votre tasse se pare d'un rouge rubis profond — comme les guirlandes qui ornent déjà le sapin. C'est Noël qui commence, une gorgée à la fois.
-En bouche, l'acidulé des canneberges danse avec la douceur sucrée des raisins, tandis que l'orange apporte sa note pétillante et fraîche. La liqueur rouge intense réchauffe les mains et le cœur, libérant des arômes de fruits d'hiver qui évoquent les marchés de Noël et les soirées au coin du feu.
-Ingrédients
-• Grains de raisin huilés (raisins, huile de tournesol)
-• Canneberges entières et sucrées (canneberges, sucre, huile de tournesol)
-• Cristaux de sucre (sucre, farine de riz, matières grasses végétales (colza), fécule de pomme de terre, colorants : E120, E160a, arôme)
-• Baies de sorbier
-• Baies d'argousier
-• Fleurs de bleuet
-• Arôme
-Conseils de préparation
-•
-Dosage : 1–2 c. à café pour 250 ml
-•
-Température : 95°C
-•
-Infusion : 8–10 minutes
-•
-Théine : Sans théine
-•
-Moment : Idéale pour vos soirées d'hiver
-Astuce gourmande : Ajoutez quelques cuillères de cette infusion dans votre vin chaud maison — les canneberges et l'orange transformeront votre breuvage en véritable élixir de fête.</t>
-        </is>
-      </c>
-      <c r="S65" s="2" t="inlineStr">
-        <is>
-          <t>Féérie d'Hiver
-Het sneeuwt buiten, en in uw keuken hangt al die feestelijke geur. U giet het borrelende water over de scharlakenrode cranberry's en de sinaasappelschillen. Vijf minuten later tooit uw kopje zich in een diep robijnrood — zoals de slingers die al de kerstboom opfleuren. Zo begint Kerstmis, slok voor slok.
-Op de tong danst de zurige frisheid van cranberry's met de zoete zachtheid van rozijnen, terwijl de sinaasappel zijn sprankelende en frisse toets brengt. De intense rode drank verwarmt handen en hart, en laat winterse fruitaroma's vrij die kerst­markten en avonden bij de haard oproepen.
-Ingrediënten
-• Geolied rozijnkorrels (rozijnen, zonnebloemolie)
-• Hele gesuikerde cranberry's (cranberry's, suiker, zonnebloemolie)
-• Suikerkristallen (suiker, rijstmeel, plantaardige vetten (koolzaad), aardappelzetmeel, kleurstoffen: E120, E160a, aroma)
-• Lijsterbessen
-• Duindoornbessen
-• Korenbloemblaadjes
-• Aroma
-Bereidingsadvies
-•
-Dosering: 1–2 tl. voor 250 ml
-•
-Temperatuur: 95°C
-•
-Trektijd: 8–10 minuten
-•
-Cafeïne: Cafeïnevrij
-•
-Moment: Ideaal voor uw winteravonden
-Lekkere tip: Voeg enkele lepels van deze infusie toe aan uw zelfgemaakte glühwein — de cranberry's en sinaasappel transformeren uw drank tot een waar feestelixer.</t>
-        </is>
-      </c>
-    </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>

</xml_diff>